<commit_message>
chore: add windows env setup script
</commit_message>
<xml_diff>
--- a/exports/products_catalog_master.xlsx
+++ b/exports/products_catalog_master.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الكتالوج الرئيسي" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="الكتالوج الرئيسي" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'الكتالوج الرئيسي'!$A$2:$N$109</definedName>
@@ -3159,7 +3159,7 @@
       </c>
       <c r="N47" s="11" t="inlineStr">
         <is>
-          <t>جملة: 380.0 ج</t>
+          <t>جملة: 260.0 ج (approved: Fares — composite box: sum of components - 5% bundle discount)</t>
         </is>
       </c>
     </row>
@@ -4672,7 +4672,7 @@
       </c>
       <c r="N74" s="11" t="inlineStr">
         <is>
-          <t>جملة: 100.0 ج</t>
+          <t>جملة: 65.0 ج (approved: Fares — graduation cap: ~28% below retail)</t>
         </is>
       </c>
     </row>
@@ -4784,7 +4784,7 @@
       </c>
       <c r="N76" s="11" t="inlineStr">
         <is>
-          <t>جملة: 200.0 ج</t>
+          <t>جملة: 115.0 ج (approved: Fares — royal shawl: ~23% below retail)</t>
         </is>
       </c>
     </row>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="N99" s="11" t="inlineStr">
         <is>
-          <t>جملة: 170.0 ج</t>
+          <t>جملة: 120.0 ج (approved: Fares — black shawl: ~20% below retail)</t>
         </is>
       </c>
     </row>

</xml_diff>